<commit_message>
07/08: align starter examples with the shipped fixtures (drift value, threshold prompts, weight allocation) and complete the readme task lists. readme and starter files only — no code or solution/demo files.
</commit_message>
<xml_diff>
--- a/07_ai-security-metrics-and-dashboarding/exercises/starter/kri_definitions.xlsx
+++ b/07_ai-security-metrics-and-dashboarding/exercises/starter/kri_definitions.xlsx
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>0.34</v>
+        <v>1.96</v>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>g ≤ 0.05% / a 0.05-0.20% / r &gt; 0.20% (rolling 7-day)</t>
+          <t>[Your response here — carry over the green/amber/red band you defined on the KRI Definitions sheet (E4).]</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>g ≤ 0.1% / a 0.1-0.5% / r &gt; 0.5%</t>
+          <t>[Your response here — carry over the green/amber/red band you defined on the KRI Definitions sheet (E5).]</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>g ≥ 90% / a 70-90% / r &lt; 70%</t>
+          <t>[Your response here — carry over the green/amber/red band you defined on the KRI Definitions sheet (E6).]</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">

</xml_diff>